<commit_message>
Rebuild foundations from S201 vectors, fix mirrored plan, add BOQ v2
- extract_s201.py reads every pile, footing and column position from the
  S201 vector PDF (734 piles, 46 F2P, 45 C1, C2, C3, F1A, F1P-1)
- model exported stage by stage from the lowest level (stages 0-2 now)
- drawing coordinates (y down the sheet) converted to world y-up; the
  previous model was a mirror image of the drawing
- site boundary taken from S202 vectors
- make_boq.py writes 01_BOQ_งานหลัก_v2.xlsx with missing items added,
  changed quantities marked, and rebar left pending design documents

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fTFw9DNpzgpK9RQnmJQ9j
</commit_message>
<xml_diff>
--- a/tongcheng-bim/out/TC-WH_BIM_QTO.xlsx
+++ b/tongcheng-bim/out/TC-WH_BIM_QTO.xlsx
@@ -580,7 +580,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>8,566</t>
+          <t>8,619</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>BOQ สมมติถมเฉลี่ย 0.50 ม. แต่แบบ A202 ระดับถนนอ้างอิงต่ำกว่าถนนรอบอาคาร 1.50 ม. ถ้าดินเดิมอยู่ที่ -1.50 ต้องถม ~8,566 ลบ.ม. (ดินเดิม -1.00 ≈ 5,593 / -0.50 ≈ 2,620) ให้ยืนยันด้วยผลสำรวจระดับ P1.2 ก่อนยื่นราคา และเสนอเป็นราคาต่อ ลบ.ม.</t>
+          <t>BOQ สมมติถมเฉลี่ย 0.50 ม. แต่แบบ A202 ระดับถนนอ้างอิงต่ำกว่าถนนรอบอาคาร 1.50 ม. ถ้าดินเดิมอยู่ที่ -1.50 ต้องถม ~8,619 ลบ.ม. (ดินเดิม -1.00 ≈ 5,625 / -0.50 ≈ 2,631) ให้ยืนยันด้วยผลสำรวจระดับ P1.2 ก่อนยื่นราคา และเสนอเป็นราคาต่อ ลบ.ม.</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>พื้นที่ 5,946 ตร.ม. ÷ 500 = 12 จุด/ชั้น × 8 ชั้น (ถมหนา 1.60 ม.) = 96 จุด</t>
+          <t>พื้นที่ 5,988 ตร.ม. ÷ 500 = 12 จุด/ชั้น × 8 ชั้น (ถมหนา 1.60 ม.) = 96 จุด</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>735</t>
+          <t>734</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>232</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>2,319</t>
+          <t>2,390</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>300</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1422,12 +1422,12 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>เส้นรอบที่ดิน (A101) ≈ 312</t>
+          <t>เส้นรอบที่ดิน (A101) ≈ 309</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>309</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1459,12 +1459,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>พื้นที่ดินตามผัง A101 ≈ 5,946</t>
+          <t>พื้นที่ดินตามผัง A101 ≈ 5,988</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>5,946</t>
+          <t>5,988</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -1600,7 +1600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J102"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1704,10 +1704,10 @@
         <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5945.69</v>
+        <v>5987.91</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>1783.706</v>
+        <v>1796.373</v>
       </c>
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="inlineStr">
@@ -1744,10 +1744,10 @@
         <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>2705.69</v>
+        <v>2747.91</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>3382.106</v>
+        <v>3434.887</v>
       </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="inlineStr">
@@ -1818,16 +1818,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>309.06</v>
+        <v>307.1</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>30.906</v>
+        <v>30.71</v>
       </c>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="inlineStr">
@@ -1997,14 +1997,14 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2.3.2 พื้นชั้นล่าง (Drop panel)</t>
+          <t>2.2.2 Drop panel F1P</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>F1P Drop panel 1.00x1.00x0.20</t>
+          <t>Drop panel F1P 1.00x1.00x0.20</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -2037,94 +2037,94 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2.1.1 เสาเข็มฐานราก</t>
+          <t>2.2.1 ฐานราก F2P</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>I26-22</t>
+          <t>F2P</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-260x260 รับฐานรากอาคาร (F2P)</t>
+          <t>ฐานราก F2P 0.60x1.50x0.80</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>2024</v>
+        <v>36.8</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>6.22</v>
+        <v>41.4</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>136.822</v>
+        <v>33.12</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>M21A</t>
+          <t>M22</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2.2.1 ฐานราก F2P</t>
+          <t>2.1.1 เสาเข็มฐานราก</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>F2P</t>
+          <t>I26-22</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>ฐานราก F2P 0.60x1.50x0.80</t>
+          <t>เสาเข็ม I-260x260 รับฐานราก F2P (หนวดกุ้ง 4-DB12-2.5 ม.)</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>36.8</v>
+        <v>2024</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>41.4</v>
+        <v>6.22</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>33.12</v>
+        <v>136.822</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>M22</t>
+          <t>M21A</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2.2.2 เสาตอม่อ คสล.</t>
+          <t>2.3.1 เสา คสล. C1</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2138,16 +2138,16 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>225.4</v>
+        <v>220.5</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>6.9</v>
+        <v>6.75</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>33.81</v>
+        <v>33.075</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="inlineStr">
@@ -2157,96 +2157,96 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2.4.1 โครงสร้างเหล็ก</t>
+          <t>2.3.2 เสา คสล. C2</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SC1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>เสาเหล็ก H250x175x44.1 kg/m</t>
+          <t>เสา คสล. C2 0.50x0.50</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>207</v>
+        <v>4.9</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>2.01</v>
+        <v>0.25</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>9.055999999999999</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>9128.700000000001</v>
-      </c>
+        <v>1.225</v>
+      </c>
+      <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>M23</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2.1.3 เสาเข็มอาคารประกอบ</t>
+          <t>2.5.1 เสาเหล็ก</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>I26-22</t>
+          <t>SC1</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-260x260 อาคารประกอบ (F1P-1)</t>
+          <t>เสาเหล็ก H250x175x44.1 kg/m</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>242</v>
+        <v>207</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.74</v>
+        <v>2.01</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>16.359</v>
-      </c>
-      <c r="H17" s="3" t="n"/>
+        <v>9.055999999999999</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>9128.700000000001</v>
+      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>M21A</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>2.2.3 ฐาน F1P-1</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2279,117 +2279,117 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>2.1.3 เสาเข็มอาคารประกอบ</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>I26-22</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>เสา คสล. C3 0.20x0.20</t>
+          <t>เสาเข็ม I-260x260 อาคารประกอบ (F1P-1)</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>27</v>
+        <v>242</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0.36</v>
+        <v>0.74</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>1.08</v>
+        <v>16.359</v>
       </c>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M21A</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2.1.3 เสาเข็มถังใต้ดิน</t>
+          <t>2.3.3 เสา คสล. C3</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>I26</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-260x260 รับถังใต้ดิน (ลดระดับ 1 ม.)</t>
+          <t>เสา คสล. C3 0.20x0.20</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>374</v>
+        <v>23.8</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>1.15</v>
+        <v>0.28</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>25.282</v>
+        <v>0.952</v>
       </c>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>M21B</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>4.3 ฐานหม้อแปลง</t>
+          <t>2.1.4 เสาเข็มถังใต้ดิน</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>I22-TR</t>
+          <t>I26</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-220x220 รับฐานหม้อแปลง</t>
+          <t>เสาเข็ม I-260x260 รับถังใต้ดิน (ลดระดับ 1 ม.)</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>132</v>
+        <v>374</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.29</v>
+        <v>1.15</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>6.389</v>
+        <v>25.282</v>
       </c>
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="inlineStr">
@@ -2399,242 +2399,242 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>4.1 งานพื้นถนนรอบอาคาร (เข็ม)</t>
+          <t>4.3.1 เข็มฐานหม้อแปลง</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>I22-22</t>
+          <t>I22-TR</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-220x220 รับพื้นถนนรอบอาคาร</t>
+          <t>เสาเข็ม I-220x220 รับฐานหม้อแปลง</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>249</v>
+        <v>6</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>5478</v>
+        <v>132</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>12.05</v>
+        <v>0.29</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>265.135</v>
+        <v>6.389</v>
       </c>
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>M21C</t>
+          <t>M21B</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>แบบ (ตำแหน่งตามระยะ 3 ม.)</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>4.1 งานพื้นถนนรอบอาคาร (ฐาน F1A)</t>
+          <t>4.1.1 เข็มพื้นถนน</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>F1A</t>
+          <t>I22-22</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>ฐาน F1A 0.60x0.60x0.30 รับพื้นรอบอาคาร</t>
+          <t>เสาเข็ม I-220x220 รับพื้นถนนรอบอาคาร</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>74.7</v>
+        <v>5104</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>89.64</v>
+        <v>11.23</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>26.892</v>
+        <v>247.034</v>
       </c>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>M41</t>
+          <t>M21C</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>2.3.1 คานคอดิน คสล.</t>
+          <t>4.1.2 ฐาน F1A</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>F1A</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>คานคอดิน B1 0.20x0.60</t>
+          <t>ฐาน F1A 0.60x0.60x0.30 รับพื้นถนน</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>47</v>
+        <v>232</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>282</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>5.64</v>
+        <v>83.52</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>33.84</v>
+        <v>25.056</v>
       </c>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>M24</t>
+          <t>M41</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>4.6.1 ฐาน 0.66 แนวเขต</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>SQ66</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>คาน B3 0.20x0.40</t>
+          <t>ฐาน 0.66x0.66 แนวเขตที่ดิน (ไม่ทราบหน้าที่)</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>37.28</v>
+        <v>4.8</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>6.97</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>2.982</v>
+        <v>2.091</v>
       </c>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M41</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ S201 (ตำแหน่ง) / หน้าที่+ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>2.3.2 พื้นชั้นล่าง คสล.</t>
+          <t>4.6.1 ฐาน 0.66 แนวเขต</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>I26-B</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>พื้น S1 คสล. หนา 0.20 ม. วางบนเสาเข็ม (TOP +0.50)</t>
+          <t>เสาเข็ม I-260x260 ใต้ฐาน 0.66 แนวเขตที่ดิน</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.2</v>
+        <v>352</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>3240</v>
+        <v>1.08</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>648</v>
+        <v>23.795</v>
       </c>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>M25</t>
+          <t>M21C</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S201 (ตำแหน่ง) / หน้าที่+ระดับรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>4.1 งานพื้นถนนรอบอาคาร S2</t>
+          <t>2.3.1 คานคอดิน คสล.</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>พื้นถนนรอบอาคาร S2 คสล. หนา 0.15 ม. (TOP ±0.00)</t>
+          <t>คานคอดิน B1 0.20x0.60</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0</v>
+        <v>282</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>2318.86</v>
+        <v>5.64</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>347.829</v>
+        <v>33.84</v>
       </c>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>M42</t>
+          <t>M24</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -2646,115 +2646,115 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>4.3 ฐานหม้อแปลง</t>
+          <t>2.5 โครงสร้างอาคารประกอบ</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>SF02</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>ฐานหม้อแปลง SF02 หนา 0.25</t>
+          <t>คาน B3 0.20x0.40</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.35</v>
+        <v>34.86</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>20.35</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>7.122</v>
+        <v>2.788</v>
       </c>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>M45</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>สมมติขนาด</t>
+          <t>สมมติตำแหน่ง</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>2.3.2 พื้นชั้นล่าง คสล.</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>พื้นอาคารห้องน้ำ S2 หนา 0.15</t>
+          <t>พื้น S1 คสล. หนา 0.20 ม. วางบนเสาเข็ม (TOP +0.50)</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>32</v>
+        <v>3240</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>4.8</v>
+        <v>648</v>
       </c>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M25</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>4.1 งานพื้นถนนรอบอาคาร S2</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>AF01</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>พื้นห้องเก็บสารเคมี AF01 หนา 0.10</t>
+          <t>พื้นถนนรอบอาคาร S2 คสล. หนา 0.15 ม. (TOP ±0.00)</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>21.84</v>
+        <v>2389.52</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>2.184</v>
+        <v>358.429</v>
       </c>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M42</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -2766,319 +2766,315 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>4.2 ทางลาดขนส่ง</t>
+          <t>4.3 ฐานหม้อแปลง</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>RAMP</t>
+          <t>SF02</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>ทางลาดขนส่งด้านเหนือ (DN) กว้าง 6.00 ม.</t>
+          <t>ฐานหม้อแปลง SF02 หนา 0.25</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>3.23</v>
+        <v>0.35</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>1.2</v>
+        <v>10.2</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>3.878</v>
+        <v>3.57</v>
       </c>
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>M43</t>
+          <t>M45</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>แบบ (ขนาดวัดจากผัง)</t>
+          <t>สมมติขนาด</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>4.2 ทางลาดขนส่ง</t>
+          <t>2.5 โครงสร้างอาคารประกอบ</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>RAMP</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>ทางลาดขนส่งด้านใต้ (DN) กว้าง 6.00 ม.</t>
+          <t>พื้นอาคารห้องน้ำ S2 หนา 0.15</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>3.53</v>
+        <v>0.15</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>1.2</v>
+        <v>19.23</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>4.235</v>
+        <v>2.885</v>
       </c>
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>M43</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>แบบ (ขนาดวัดจากผัง)</t>
+          <t>สมมติตำแหน่ง</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>4.4 ถังเก็บน้ำใต้ดิน</t>
+          <t>2.5 โครงสร้างอาคารประกอบ</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>UGT</t>
+          <t>AF01</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>ถังเก็บน้ำใต้ดิน - พื้น หนา 0.25 (BF -2.85)</t>
+          <t>พื้นห้องเก็บสารเคมี AF01 หนา 0.10</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>87</v>
+        <v>24.14</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>21.75</v>
+        <v>2.414</v>
       </c>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>M26</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>แบบ (ขนาดวัดจากผัง)</t>
+          <t>แบบ</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>4.4 ถังเก็บน้ำใต้ดิน</t>
+          <t>4.2 ทางลาดขนส่ง</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>UGT</t>
+          <t>RAMP</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ถังเก็บน้ำใต้ดิน - ผนัง คสล. หนา 0.25</t>
+          <t>ทางลาดขนส่งด้านเหนือ (DN) กว้าง 6.00 ม.</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>3.23</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>58.06</v>
+        <v>1.2</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>23.398</v>
+        <v>3.878</v>
       </c>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>M26</t>
+          <t>M43</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (ขนาดวัดจากผัง)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>4.4 ถังเก็บน้ำใต้ดิน</t>
+          <t>4.2 ทางลาดขนส่ง</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>UGT</t>
+          <t>RAMP</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>ถังเก็บน้ำใต้ดิน - ฝา หนา 0.15</t>
+          <t>ทางลาดขนส่งด้านใต้ (DN) กว้าง 6.00 ม.</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.15</v>
+        <v>3.53</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>87</v>
+        <v>1.2</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>13.05</v>
+        <v>4.235</v>
       </c>
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>M26</t>
+          <t>M43</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (ขนาดวัดจากผัง)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>4.5 รางระบายน้ำพร้อมฝาปิด</t>
+          <t>4.4 ถังเก็บน้ำใต้ดิน</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>DR</t>
+          <t>UGT</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>รางระบายน้ำ คสล. พร้อมฝาปิด 0.40x0.50</t>
+          <t>ถังเก็บน้ำใต้ดิน - พื้น หนา 0.25 (BF -2.85)</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>301.73</v>
+        <v>0.25</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>0.8</v>
+        <v>80.36</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>60.346</v>
+        <v>20.089</v>
       </c>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>M46</t>
+          <t>M26</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>แบบ (แนวโดยประมาณ)</t>
+          <t>แบบ (ขนาดวัดจากผัง)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>3.6 ชั้นลอย (โครงเหล็ก)</t>
+          <t>4.4 ถังเก็บน้ำใต้ดิน</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>UGT</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>เสาชั้นลอย H250x250x66.5 kg/m</t>
+          <t>ถังเก็บน้ำใต้ดิน - ผนัง คสล. หนา 0.25</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>100.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>2.25</v>
+        <v>60.61</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="H37" s="3" t="n">
-        <v>6703.2</v>
-      </c>
+        <v>22.969</v>
+      </c>
+      <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>M35</t>
+          <t>M26</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>3.6 ชั้นลอย (โครงเหล็ก)</t>
+          <t>4.4 ถังเก็บน้ำใต้ดิน</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>UGT</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>คานชั้นลอย H200x100 (สมมติ)</t>
+          <t>ถังเก็บน้ำใต้ดิน - ฝา หนา 0.15</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>245</v>
+        <v>0.15</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>0.28</v>
+        <v>80.36</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="H38" s="3" t="n">
-        <v>5218.5</v>
-      </c>
+        <v>12.053</v>
+      </c>
+      <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>M35</t>
+          <t>M26</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
@@ -3090,72 +3086,74 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>3.6 ชั้นลอย (พื้น)</t>
+          <t>4.5 รางระบายน้ำพร้อมฝาปิด</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>F8</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>พื้นชั้นลอย F8 (TOP +3.30)</t>
+          <t>รางระบายน้ำ คสล. พร้อมฝาปิด 0.40x0.50</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0.03</v>
+        <v>300.09</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>306</v>
+        <v>2.2</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>9.18</v>
+        <v>60.018</v>
       </c>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>M35</t>
+          <t>M46</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ (แนวโดยประมาณ)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>3.6 ชั้นลอย (บันได)</t>
+          <t>3.6 ชั้นลอย (โครงเหล็ก)</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>ST</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>บันไดชั้นลอย กว้าง 1.40 ม.</t>
+          <t>เสาชั้นลอย H250x250x66.5 kg/m</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>5.05</v>
+        <v>100.8</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>0.21</v>
+        <v>2.25</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="H40" s="3" t="n"/>
+        <v>6.3</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>6703.2</v>
+      </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
           <t>M35</t>
@@ -3163,133 +3161,129 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>แบบ (ตำแหน่ง DN)</t>
+          <t>แบบ</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2.4.1 โครงสร้างเหล็ก (โครงถัก)</t>
+          <t>3.6 ชั้นลอย (โครงเหล็ก)</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว A - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>คานชั้นลอย H200x100 (สมมติ)</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>60.52</v>
+        <v>245</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0.04</v>
+        <v>0.28</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>1.18</v>
+        <v>4.9</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>907.8</v>
+        <v>5218.5</v>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>M32</t>
+          <t>M35</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>2.4.1 โครงสร้างเหล็ก (โครงถัก)</t>
+          <t>3.6 ชั้นลอย (พื้น)</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>F8</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว A - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>พื้นชั้นลอย F8 (TOP +3.30)</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>60.13</v>
+        <v>0.03</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>0.04</v>
+        <v>306</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>1.173</v>
-      </c>
-      <c r="H42" s="3" t="n">
-        <v>902</v>
-      </c>
+        <v>9.18</v>
+      </c>
+      <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>M32</t>
+          <t>M35</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>แบบ</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2.4.1 โครงสร้างเหล็ก (โครงถัก)</t>
+          <t>3.6 ชั้นลอย (บันได)</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว A - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>บันไดชั้นลอย กว้าง 1.40 ม.</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>82.95</v>
+        <v>5.05</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>0.21</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.415</v>
-      </c>
-      <c r="H43" s="3" t="n">
-        <v>336.8</v>
-      </c>
+        <v>1.06</v>
+      </c>
+      <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>M32</t>
+          <t>M35</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (ตำแหน่ง DN)</t>
         </is>
       </c>
     </row>
@@ -3301,28 +3295,28 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว A - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว A - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -3331,7 +3325,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -3343,28 +3337,28 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว B - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว A - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F45" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
@@ -3385,28 +3379,28 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว B - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว A - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -3415,7 +3409,7 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -3432,23 +3426,23 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว B - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว A - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
@@ -3469,28 +3463,28 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว B - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว B - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -3499,7 +3493,7 @@
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -3511,28 +3505,28 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว C - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว B - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F49" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
@@ -3553,28 +3547,28 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว C - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว B - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
@@ -3583,7 +3577,7 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -3600,23 +3594,23 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว C - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว B - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
@@ -3637,28 +3631,28 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว C - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว C - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
@@ -3667,7 +3661,7 @@
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -3679,28 +3673,28 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว D - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว C - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D53" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F53" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
@@ -3721,28 +3715,28 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว D - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว C - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
@@ -3751,7 +3745,7 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -3768,23 +3762,23 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว D - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว C - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
@@ -3805,28 +3799,28 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว D - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว D - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
@@ -3835,7 +3829,7 @@
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -3847,28 +3841,28 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว E - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว D - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D57" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F57" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
@@ -3889,28 +3883,28 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว E - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว D - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
@@ -3919,7 +3913,7 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -3936,23 +3930,23 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว E - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว D - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
@@ -3973,28 +3967,28 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว E - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว E - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
@@ -4003,7 +3997,7 @@
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -4015,28 +4009,28 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว F - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว E - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D61" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F61" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
@@ -4057,28 +4051,28 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว F - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว E - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
@@ -4087,7 +4081,7 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -4104,23 +4098,23 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว F - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว E - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
@@ -4141,28 +4135,28 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว F - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว F - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
@@ -4171,7 +4165,7 @@
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -4183,28 +4177,28 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว G - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว F - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D65" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F65" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
@@ -4225,28 +4219,28 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว G - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว F - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
@@ -4255,7 +4249,7 @@
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -4272,23 +4266,23 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว G - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว F - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
@@ -4309,28 +4303,28 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว G - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว G - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
@@ -4339,7 +4333,7 @@
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -4351,28 +4345,28 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว H - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว G - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D69" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F69" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
@@ -4393,28 +4387,28 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว H - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว G - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G70" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
@@ -4423,7 +4417,7 @@
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -4440,23 +4434,23 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว H - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว G - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
@@ -4477,28 +4471,28 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว H - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว H - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G72" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
@@ -4507,7 +4501,7 @@
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -4519,28 +4513,28 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว I - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว H - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D73" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
@@ -4561,28 +4555,28 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว I - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว H - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
@@ -4591,7 +4585,7 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -4608,23 +4602,23 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว I - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว H - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
@@ -4645,28 +4639,28 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว I - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว I - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
@@ -4675,7 +4669,7 @@
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
@@ -4687,28 +4681,28 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>TR-TC</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว J - คอร์ดบน 2C-150x65x20x3.2</t>
+          <t>โครงถัก (Truss) แนว I - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D77" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>60.52</v>
+        <v>60.13</v>
       </c>
       <c r="F77" s="3" t="n">
         <v>0.04</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>1.18</v>
+        <v>1.173</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>907.8</v>
+        <v>902</v>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
@@ -4729,28 +4723,28 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>TR-BC</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก (Truss) แนว J - คอร์ดล่าง 2C-150x65x20x3.2</t>
+          <t>โครงถัก แนว I - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>60.13</v>
+        <v>82.95</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>1.173</v>
+        <v>0.415</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>902</v>
+        <v>336.8</v>
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
@@ -4759,7 +4753,7 @@
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>แบบ (หน้าตัดสมมติ)</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
@@ -4776,23 +4770,23 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว J - ค้ำตั้ง C-100x50x20x2.3</t>
+          <t>โครงถัก แนว I - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>82.95</v>
+        <v>100.21</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>0.415</v>
+        <v>0.501</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>336.8</v>
+        <v>406.8</v>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
@@ -4813,28 +4807,28 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>TR-W</t>
+          <t>TR-TC</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>โครงถัก แนว J - ค้ำทแยง C-100x50x20x2.3</t>
+          <t>โครงถัก (Truss) แนว J - คอร์ดบน 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>100.21</v>
+        <v>60.52</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>0.501</v>
+        <v>1.18</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>406.8</v>
+        <v>907.8</v>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
@@ -4843,82 +4837,82 @@
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>2.4.1 โครงสร้างเหล็ก (แป)</t>
+          <t>2.4.1 โครงสร้างเหล็ก (โครงถัก)</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>TR-BC</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>แป C-125x50x20x3.2</t>
+          <t>โครงถัก (Truss) แนว J - คอร์ดล่าง 2C-150x65x20x3.2</t>
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>2730</v>
+        <v>60.13</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>0.31</v>
+        <v>0.04</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>17.063</v>
+        <v>1.173</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>16734.9</v>
+        <v>902</v>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>M33</t>
+          <t>M32</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ (หน้าตัดสมมติ)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>2.4.1 โครงสร้างเหล็ก (ค้ำยัน)</t>
+          <t>2.4.1 โครงสร้างเหล็ก (โครงถัก)</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>ค้ำยันหลังคา RB12 + Turnbuckle</t>
+          <t>โครงถัก แนว J - ค้ำตั้ง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>340.88</v>
+        <v>82.95</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>0.01</v>
+        <v>0.21</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>0.049</v>
+        <v>0.415</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>302.7</v>
+        <v>336.8</v>
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
@@ -4934,37 +4928,37 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>2.4.1 โครงสร้างเหล็ก (แปผนัง)</t>
+          <t>2.4.1 โครงสร้างเหล็ก (โครงถัก)</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>TR-W</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>แปผนัง (Girt) C-125x50x20x3.2</t>
+          <t>โครงถัก แนว J - ค้ำทแยง C-100x50x20x2.3</t>
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>684</v>
+        <v>100.21</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>4.275</v>
+        <v>0.501</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>4192.9</v>
+        <v>406.8</v>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>M33</t>
+          <t>M32</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
@@ -4976,150 +4970,156 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (มุงหลังคา)</t>
+          <t>2.4.1 โครงสร้างเหล็ก (แป)</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>หลังคาเมทัลชีท หนา 0.47 มม. + ฉนวน PU 25 มม.</t>
+          <t>แป C-125x50x20x3.2</t>
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>0.1</v>
+        <v>2730</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>3.09</v>
+        <v>0.31</v>
       </c>
       <c r="G84" s="3" t="n">
-        <v>169.753</v>
-      </c>
-      <c r="H84" s="3" t="n"/>
+        <v>17.063</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>16734.9</v>
+      </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>M34</t>
+          <t>M33</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>สมมติสเปค</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (Jack roof)</t>
+          <t>2.4.1 โครงสร้างเหล็ก (ค้ำยัน)</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>JR</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Jack roof กว้าง 6.00 ม. (สัน +15.25)</t>
+          <t>ค้ำยันหลังคา RB12 + Turnbuckle</t>
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>0.05</v>
+        <v>340.88</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>0.3</v>
+        <v>0.01</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="H85" s="3" t="n"/>
+        <v>0.049</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>302.7</v>
+      </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>M34</t>
+          <t>M32</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (Jack roof)</t>
+          <t>2.4.1 โครงสร้างเหล็ก (แปผนัง)</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>JR-L</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>ช่องระบายอากาศ Jack roof (ตะแกรง)</t>
+          <t>แปผนัง (Girt) C-125x50x20x3.2</t>
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>2.89</v>
+        <v>684</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>0.17</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>7.283</v>
-      </c>
-      <c r="H86" s="3" t="n"/>
+        <v>4.275</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>4192.9</v>
+      </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>M34</t>
+          <t>M33</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (รางน้ำ)</t>
+          <t>3.1 หลังคาและผนังภายนอก (มุงหลังคา)</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>GU</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30</t>
+          <t>หลังคาเมทัลชีท หนา 0.47 มม. + ฉนวน PU 25 มม.</t>
         </is>
       </c>
       <c r="D87" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>33</v>
+        <v>3.09</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>9.9</v>
+        <v>169.753</v>
       </c>
       <c r="H87" s="3" t="n"/>
       <c r="I87" s="3" t="inlineStr">
@@ -5129,37 +5129,37 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>สมมติสเปค</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (ท่อน้ำฝน)</t>
+          <t>3.1 หลังคาและผนังภายนอก (Jack roof)</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>DP</t>
+          <t>JR</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>ท่อระบายน้ำฝน PVC Ø4"</t>
+          <t>Jack roof กว้าง 6.00 ม. (สัน +15.25)</t>
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>97.5</v>
+        <v>0.05</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="G88" s="3" t="n">
-        <v>0.975</v>
+        <v>12.6</v>
       </c>
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="inlineStr">
@@ -5169,327 +5169,327 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>สมมติ</t>
+          <t>แบบ</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>3.2 ผนังก่ออิฐฉาบปูน</t>
+          <t>3.1 หลังคาและผนังภายนอก (Jack roof)</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>JR-L</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ฉาบปูน 2 ด้าน + ทาสี (ถึง +4.50)</t>
+          <t>ช่องระบายอากาศ Jack roof (ตะแกรง)</t>
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>24</v>
+        <v>2.89</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>435.6</v>
+        <v>0.17</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>130.14</v>
+        <v>7.283</v>
       </c>
       <c r="H89" s="3" t="n"/>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>M36</t>
+          <t>M34</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (ตาม A202)</t>
+          <t>แบบ</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
+          <t>3.1 หลังคาและผนังภายนอก (รางน้ำ)</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>GU</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>ผนังเมทัลชีท (ด้านจั่ว) +5.20 ถึงหลังคา</t>
+          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30</t>
         </is>
       </c>
       <c r="D90" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>837</v>
+        <v>33</v>
       </c>
       <c r="G90" s="3" t="n">
-        <v>25.11</v>
+        <v>9.9</v>
       </c>
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>M37</t>
+          <t>M34</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>แบบ A202</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
+          <t>3.1 หลังคาและผนังภายนอก (ท่อน้ำฝน)</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>DP</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>ผนังเมทัลชีท (ด้านชายคา) +5.20 ถึง +10.00</t>
+          <t>ท่อระบายน้ำฝน PVC Ø4"</t>
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>10</v>
+        <v>97.5</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>16.26</v>
+        <v>0.975</v>
       </c>
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>M37</t>
+          <t>M34</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>แบบ A202</t>
+          <t>สมมติ</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
+          <t>3.2 ผนังก่ออิฐฉาบปูน</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>RD1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดเหนือ)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ฉาบปูน 2 ด้าน + ทาสี (ถึง +4.50)</t>
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>24</v>
+        <v>435.6</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>2.88</v>
+        <v>130.14</v>
       </c>
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>M38</t>
+          <t>M36</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>สมมติขนาด</t>
+          <t>สมมติ (ตาม A202)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
+          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>RD2</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดใต้)</t>
+          <t>ผนังเมทัลชีท (ด้านจั่ว) +5.20 ถึงหลังคา</t>
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>24</v>
+        <v>837</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>2.88</v>
+        <v>25.11</v>
       </c>
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>M38</t>
+          <t>M37</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>สมมติขนาด</t>
+          <t>แบบ A202</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ - ผนังก่ออิฐ</t>
+          <t>ผนังเมทัลชีท (ด้านชายคา) +5.20 ถึง +10.00</t>
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>11.4</v>
+        <v>10</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>23.37</v>
+        <v>0.3</v>
       </c>
       <c r="G94" s="3" t="n">
-        <v>6.84</v>
+        <v>16.26</v>
       </c>
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M37</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
+          <t>แบบ A202</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>RD1</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ - หลังคา/ฝ้า</t>
+          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดเหนือ)</t>
         </is>
       </c>
       <c r="D95" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>0.1</v>
+        <v>4</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>3.2</v>
+        <v>2.88</v>
       </c>
       <c r="H95" s="3" t="n"/>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
+          <t>สมมติขนาด</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>RD2</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - ผนังก่ออิฐ</t>
+          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดใต้)</t>
         </is>
       </c>
       <c r="D96" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E96" s="3" t="n">
-        <v>11.2</v>
-      </c>
       <c r="F96" s="3" t="n">
-        <v>20.94</v>
+        <v>24</v>
       </c>
       <c r="G96" s="3" t="n">
-        <v>5.398</v>
+        <v>2.88</v>
       </c>
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>สมมติขนาด</t>
         </is>
       </c>
     </row>
@@ -5501,25 +5501,25 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - หลังคา/ฝ้า</t>
+          <t>อาคารห้องน้ำ - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>0.1</v>
+        <v>11.4</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>21.84</v>
+        <v>14.27</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>2.184</v>
+        <v>5.932</v>
       </c>
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
         </is>
       </c>
     </row>
@@ -5541,35 +5541,35 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. - ผนังก่ออิฐ</t>
+          <t>อาคารห้องน้ำ - หลังคา/ฝ้า</t>
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>11.2</v>
+        <v>0.1</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>33.77</v>
+        <v>19.23</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>5.001</v>
+        <v>1.923</v>
       </c>
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
         </is>
       </c>
     </row>
@@ -5581,30 +5581,30 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>CHEM</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. - หลังคา/ฝ้า</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>0.1</v>
+        <v>11.2</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>17.79</v>
+        <v>23.04</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>1.779</v>
+        <v>5.615</v>
       </c>
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
@@ -5621,35 +5621,35 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>CHEM</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (รอแบบ) - ผนังก่ออิฐ</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - หลังคา/ฝ้า</t>
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>11.2</v>
+        <v>0.1</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>72.63</v>
+        <v>24.14</v>
       </c>
       <c r="G100" s="3" t="n">
-        <v>9.446999999999999</v>
+        <v>2.414</v>
       </c>
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (A101)</t>
+          <t>แบบ A101</t>
         </is>
       </c>
     </row>
@@ -5661,25 +5661,25 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (รอแบบ) - หลังคา/ฝ้า</t>
+          <t>ห้อง MDB 17.79 ตร.ม. - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>0.1</v>
+        <v>11.2</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>51.48</v>
+        <v>33.77</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>5.148</v>
+        <v>5.001</v>
       </c>
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="inlineStr">
@@ -5689,24 +5689,24 @@
       </c>
       <c r="J101" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (A101)</t>
+          <t>แบบ A101</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>4.1 งานพื้นถนนรอบอาคาร</t>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>AF01</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>พื้นทางเท้า/ลานหน้าห้องเก็บสารเคมี AF01</t>
+          <t>ห้อง MDB 17.79 ตร.ม. - หลังคา/ฝ้า</t>
         </is>
       </c>
       <c r="D102" s="3" t="n">
@@ -5716,18 +5716,138 @@
         <v>0.1</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>16.74</v>
+        <v>17.79</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>1.674</v>
+        <v>1.779</v>
       </c>
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="inlineStr">
         <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>แบบ A101</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>ห้องประกอบแนวกริด A (รอแบบ) - ผนังก่ออิฐ</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E103" s="3" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>72.63</v>
+      </c>
+      <c r="G103" s="3" t="n">
+        <v>9.446999999999999</v>
+      </c>
+      <c r="H103" s="3" t="n"/>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>สมมติ (A101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>ห้องประกอบแนวกริด A (รอแบบ) - หลังคา/ฝ้า</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>51.48</v>
+      </c>
+      <c r="G104" s="3" t="n">
+        <v>5.148</v>
+      </c>
+      <c r="H104" s="3" t="n"/>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>สมมติ (A101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>4.1 งานพื้นถนนรอบอาคาร</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>AF01</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>พื้นทางเท้า/ลานหน้าห้องเก็บสารเคมี AF01</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F105" s="3" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="G105" s="3" t="n">
+        <v>1.674</v>
+      </c>
+      <c r="H105" s="3" t="n"/>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
           <t>M42</t>
         </is>
       </c>
-      <c r="J102" s="3" t="inlineStr">
+      <c r="J105" s="3" t="inlineStr">
         <is>
           <t>สมมติตำแหน่ง</t>
         </is>
@@ -6184,7 +6304,7 @@
         </is>
       </c>
       <c r="K11" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -6411,7 +6531,7 @@
         </is>
       </c>
       <c r="K16" s="3" t="n">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="17">
@@ -6548,7 +6668,7 @@
         </is>
       </c>
       <c r="K19" s="3" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -6591,7 +6711,7 @@
         </is>
       </c>
       <c r="K20" s="3" t="n">
-        <v>407</v>
+        <v>360</v>
       </c>
     </row>
     <row r="21">
@@ -6634,7 +6754,7 @@
         </is>
       </c>
       <c r="K21" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -6724,7 +6844,7 @@
         </is>
       </c>
       <c r="K23" s="3" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -6771,7 +6891,7 @@
         </is>
       </c>
       <c r="K24" s="3" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -6818,7 +6938,7 @@
         </is>
       </c>
       <c r="K25" s="3" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -6865,7 +6985,7 @@
         </is>
       </c>
       <c r="K26" s="3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -6912,7 +7032,7 @@
         </is>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -6959,7 +7079,7 @@
         </is>
       </c>
       <c r="K28" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -7002,7 +7122,7 @@
         </is>
       </c>
       <c r="K29" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -7045,7 +7165,7 @@
         </is>
       </c>
       <c r="K30" s="3" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -7088,7 +7208,7 @@
         </is>
       </c>
       <c r="K31" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -7131,7 +7251,7 @@
         </is>
       </c>
       <c r="K32" s="3" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -7178,7 +7298,7 @@
         </is>
       </c>
       <c r="K33" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -7221,7 +7341,7 @@
         </is>
       </c>
       <c r="K34" s="3" t="n">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="35">
@@ -7264,7 +7384,7 @@
         </is>
       </c>
       <c r="K35" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -7307,7 +7427,7 @@
         </is>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -7350,7 +7470,7 @@
         </is>
       </c>
       <c r="K37" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -7393,7 +7513,7 @@
         </is>
       </c>
       <c r="K38" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -7553,13 +7673,13 @@
         <v>-1.5</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3382</v>
+        <v>3435</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>5184</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>8566</v>
+        <v>8619</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
@@ -7572,13 +7692,13 @@
         <v>-1</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>2029</v>
+        <v>2061</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>3564</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5593</v>
+        <v>5625</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
@@ -7591,13 +7711,13 @@
         <v>-0.5</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>676</v>
+        <v>687</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>1944</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2620</v>
+        <v>2631</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Model all construction stages bottom-up with stage selector
- annex beams B3 at S202 levels (toilet +0.50, chemical room road level)
- AF01 floors per S6.1, personnel doors at A101 tag positions
- viewer can show stages 0-8 cumulatively, latest stage highlighted

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fTFw9DNpzgpK9RQnmJQ9j
</commit_message>
<xml_diff>
--- a/tongcheng-bim/out/TC-WH_BIM_QTO.xlsx
+++ b/tongcheng-bim/out/TC-WH_BIM_QTO.xlsx
@@ -1600,7 +1600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2646,7 +2646,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>2.3.5 คาน B3</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -2660,16 +2660,16 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>34.86</v>
+        <v>38.87</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.64</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>2.788</v>
+        <v>3.11</v>
       </c>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ S202 (ตำแหน่ง+ระดับ)</t>
         </is>
       </c>
     </row>
@@ -2746,10 +2746,10 @@
         <v>0</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>2389.52</v>
+        <v>2389.58</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>358.429</v>
+        <v>358.438</v>
       </c>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="inlineStr">
@@ -2806,30 +2806,30 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>2.4.2 พื้น AF01</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>AF01</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>พื้นอาคารห้องน้ำ S2 หนา 0.15</t>
+          <t>พื้นอาคารห้องน้ำ AF01 หนา 0.10 (TOP +0.50)</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>19.23</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>2.885</v>
+        <v>1.923</v>
       </c>
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="inlineStr">
@@ -2839,14 +2839,14 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง</t>
+          <t>แบบ S202/S6.1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2.5 โครงสร้างอาคารประกอบ</t>
+          <t>2.4.2 พื้น AF01</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>พื้นห้องเก็บสารเคมี AF01 หนา 0.10</t>
+          <t>พื้นห้องเก็บสารเคมี AF01 หนา 0.10 (TOP ±0.00)</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>แบบ S202/S6.1</t>
         </is>
       </c>
     </row>
@@ -2903,13 +2903,13 @@
         <v>1</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>3.23</v>
+        <v>3.22</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>1.2</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>3.878</v>
+        <v>3.866</v>
       </c>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="inlineStr">
@@ -5496,80 +5496,80 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4.2 ประตู D1/D2/D4</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ - ผนังก่ออิฐ</t>
+          <t>ประตู D1 (ตำแหน่งจาก A101 ขนาดรอตารางประตู)</t>
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>11.4</v>
+        <v>6.3</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>14.27</v>
+        <v>2.77</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>5.932</v>
+        <v>1.008</v>
       </c>
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
+          <t>แบบ A101 (ตำแหน่ง) / ขนาดสมมติ</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4.2 ประตู D1/D2/D4</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ - หลังคา/ฝ้า</t>
+          <t>ประตู D2 (ตำแหน่งจาก A101 ขนาดรอตารางประตู)</t>
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>0.1</v>
+        <v>4.2</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>19.23</v>
+        <v>7.56</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>1.923</v>
+        <v>1.21</v>
       </c>
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
+          <t>แบบ A101 (ตำแหน่ง) / ขนาดสมมติ</t>
         </is>
       </c>
     </row>
@@ -5581,25 +5581,25 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - ผนังก่ออิฐ</t>
+          <t>อาคารห้องน้ำ - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D99" s="3" t="n">
         <v>4</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>11.2</v>
+        <v>10</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>23.04</v>
+        <v>12.52</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>5.615</v>
+        <v>5.204</v>
       </c>
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="inlineStr">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
         </is>
       </c>
     </row>
@@ -5621,12 +5621,12 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - หลังคา/ฝ้า</t>
+          <t>อาคารห้องน้ำ - หลังคา/ฝ้า</t>
         </is>
       </c>
       <c r="D100" s="3" t="n">
@@ -5636,10 +5636,10 @@
         <v>0.1</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>24.14</v>
+        <v>19.23</v>
       </c>
       <c r="G100" s="3" t="n">
-        <v>2.414</v>
+        <v>1.923</v>
       </c>
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="inlineStr">
@@ -5649,7 +5649,7 @@
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
         </is>
       </c>
     </row>
@@ -5661,30 +5661,30 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>CHEM</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. - ผนังก่ออิฐ</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D101" s="3" t="n">
         <v>4</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>11.2</v>
+        <v>13.2</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>33.77</v>
+        <v>27.16</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>5.001</v>
+        <v>6.618</v>
       </c>
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J101" s="3" t="inlineStr">
@@ -5701,12 +5701,12 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>CHEM</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. - หลังคา/ฝ้า</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - หลังคา/ฝ้า</t>
         </is>
       </c>
       <c r="D102" s="3" t="n">
@@ -5716,15 +5716,15 @@
         <v>0.1</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>17.79</v>
+        <v>24.14</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>1.779</v>
+        <v>2.414</v>
       </c>
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J102" s="3" t="inlineStr">
@@ -5741,12 +5741,12 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (รอแบบ) - ผนังก่ออิฐ</t>
+          <t>ห้อง MDB 17.79 ตร.ม. - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D103" s="3" t="n">
@@ -5756,10 +5756,10 @@
         <v>11.2</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>72.63</v>
+        <v>33.77</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>9.446999999999999</v>
+        <v>5.001</v>
       </c>
       <c r="H103" s="3" t="n"/>
       <c r="I103" s="3" t="inlineStr">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (A101)</t>
+          <t>แบบ A101</t>
         </is>
       </c>
     </row>
@@ -5781,12 +5781,12 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (รอแบบ) - หลังคา/ฝ้า</t>
+          <t>ห้อง MDB 17.79 ตร.ม. - หลังคา/ฝ้า</t>
         </is>
       </c>
       <c r="D104" s="3" t="n">
@@ -5796,10 +5796,10 @@
         <v>0.1</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>51.48</v>
+        <v>17.79</v>
       </c>
       <c r="G104" s="3" t="n">
-        <v>5.148</v>
+        <v>1.779</v>
       </c>
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="inlineStr">
@@ -5809,45 +5809,125 @@
       </c>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (A101)</t>
+          <t>แบบ A101</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>4.1 งานพื้นถนนรอบอาคาร</t>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>AF01</t>
+          <t>RM</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>พื้นทางเท้า/ลานหน้าห้องเก็บสารเคมี AF01</t>
+          <t>ห้องประกอบแนวกริด A (รอแบบ) - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>0.1</v>
+        <v>11.2</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>16.74</v>
+        <v>72.63</v>
       </c>
       <c r="G105" s="3" t="n">
-        <v>1.674</v>
+        <v>9.446999999999999</v>
       </c>
       <c r="H105" s="3" t="n"/>
       <c r="I105" s="3" t="inlineStr">
         <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>สมมติ (A101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>ห้องประกอบแนวกริด A (รอแบบ) - หลังคา/ฝ้า</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F106" s="3" t="n">
+        <v>51.48</v>
+      </c>
+      <c r="G106" s="3" t="n">
+        <v>5.148</v>
+      </c>
+      <c r="H106" s="3" t="n"/>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>สมมติ (A101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>4.1 งานพื้นถนนรอบอาคาร</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>AF01</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>พื้นทางเท้า/ลานหน้าห้องเก็บสารเคมี AF01</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="G107" s="3" t="n">
+        <v>1.674</v>
+      </c>
+      <c r="H107" s="3" t="n"/>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
           <t>M42</t>
         </is>
       </c>
-      <c r="J105" s="3" t="inlineStr">
+      <c r="J107" s="3" t="inlineStr">
         <is>
           <t>สมมติตำแหน่ง</t>
         </is>
@@ -6668,7 +6748,7 @@
         </is>
       </c>
       <c r="K19" s="3" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20">
@@ -6711,7 +6791,7 @@
         </is>
       </c>
       <c r="K20" s="3" t="n">
-        <v>360</v>
+        <v>407</v>
       </c>
     </row>
     <row r="21">
@@ -6754,7 +6834,7 @@
         </is>
       </c>
       <c r="K21" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -6844,7 +6924,7 @@
         </is>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24">
@@ -6891,7 +6971,7 @@
         </is>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="25">
@@ -6938,7 +7018,7 @@
         </is>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26">
@@ -6985,7 +7065,7 @@
         </is>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27">
@@ -7032,7 +7112,7 @@
         </is>
       </c>
       <c r="K27" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -7079,7 +7159,7 @@
         </is>
       </c>
       <c r="K28" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -7122,7 +7202,7 @@
         </is>
       </c>
       <c r="K29" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -7165,7 +7245,7 @@
         </is>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31">
@@ -7208,7 +7288,7 @@
         </is>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32">
@@ -7251,7 +7331,7 @@
         </is>
       </c>
       <c r="K32" s="3" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
@@ -7298,7 +7378,7 @@
         </is>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -7384,7 +7464,7 @@
         </is>
       </c>
       <c r="K35" s="3" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36">
@@ -7427,7 +7507,7 @@
         </is>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -7470,7 +7550,7 @@
         </is>
       </c>
       <c r="K37" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -7513,7 +7593,7 @@
         </is>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
Complete BOQ v2 missing items and add second-pass check
- add missing items: adjacent-building survey, backfill, crane/man lift,
  pile splices, slab PE sheet and joints, base-plate grout, mezzanine
  guardrail, bird screen, D1 door steps, road sub-base, tank breakdown,
  rainwater pipes, category 5 building services as provisional sums
- perimeter walls per bay: masonry to +4.35, lintel +4.35..+4.50,
  tie beam at door head, stiffener columns, corner forming before plaster
  (per-wall sheet), plaster/paint incl. exposed RC columns
- F2P confirmed 46 footings; steel columns H250x175 corrected to 46
- second-pass check sheet compares quantities with S201/S202 vectors,
  schedule tables and the model; flags order, units and missing quantities

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fTFw9DNpzgpK9RQnmJQ9j
</commit_message>
<xml_diff>
--- a/tongcheng-bim/out/TC-WH_BIM_QTO.xlsx
+++ b/tongcheng-bim/out/TC-WH_BIM_QTO.xlsx
@@ -701,7 +701,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>แบบนับรวมฐาน F1P-1 เข็มเดี่ยว 11 ต้น (อาคารประกอบ) และ F2P 47 ฐาน; โมเดลวาง F2P ได้ 46 ฐาน = 92 + 11 = 103</t>
+          <t>F2P 46 ฐาน x 2 = 92 ต้น (ผู้ว่าจ้างยืนยัน) + F1P-1 11 ต้น = 103; ตาราง S2 = 105 (นับจาก F2P 47 ฐาน)</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>47 (ปริมาตร 33.12 ลบ.ม. = 46 ฐาน)</t>
+          <t>ผัง S201 46 / ตาราง S1.1 47</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -879,14 +879,14 @@
           <t>46</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>สมมติ/ตรวจ</t>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>ตรง</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>ตารางนับ 47 แต่ปริมาตรเท่ากับ 46 ฐาน (0.72 ลบ.ม./ฐาน) และผัง S201 นับได้ 46 → ตรวจหาฐานซ้อนใน Revit</t>
+          <t>ผู้ว่าจ้างยืนยัน 46 ฐาน (เสา C1 45 + C2 1, เข็ม 92 ต้น) ตาราง S1.1 นับ 47 ผิด เสาเหล็ก H250x175 จึงเป็น 46 ต้น</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>868</t>
+          <t>784</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -1600,7 +1600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5256,7 +5256,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>3.2 ผนังก่ออิฐฉาบปูน</t>
+          <t>3.2.1 ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -5266,20 +5266,20 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ฉาบปูน 2 ด้าน + ทาสี (ถึง +4.50)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 +0.50 ถึง +4.35 (ผนังแนวกริด A)</t>
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>24</v>
+        <v>34.65</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>435.6</v>
+        <v>197.5</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>130.14</v>
+        <v>29.626</v>
       </c>
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="inlineStr">
@@ -5289,487 +5289,487 @@
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (ตาม A202)</t>
+          <t>ผู้ว่าจ้างกำหนดระดับ / A202</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
+          <t>3.2.3 คานทับหลัง</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>ผนังเมทัลชีท (ด้านจั่ว) +5.20 ถึงหลังคา</t>
+          <t>คานทับหลัง คสล. 0.15x0.15 ม. +4.35..+4.50</t>
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>0</v>
+        <v>205.2</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>837</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>25.11</v>
+        <v>4.617</v>
       </c>
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>M37</t>
+          <t>M36</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>แบบ A202</t>
+          <t>ผู้ว่าจ้างกำหนดระดับ</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
+          <t>3.2.4 คานเอ็น</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>ผนังเมทัลชีท (ด้านชายคา) +5.20 ถึง +10.00</t>
+          <t>คานเอ็น คสล. 0.15x0.10 ม. ระดับหลังประตู +2.60</t>
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>10</v>
+        <v>205.2</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>0.3</v>
+        <v>0.54</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>16.26</v>
+        <v>3.078</v>
       </c>
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>M37</t>
+          <t>M36</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>แบบ A202</t>
+          <t>สมมติตามมาตรฐานผนังก่อ (สูง &gt; 3 ม.)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
+          <t>3.2.5 เสาเอ็น</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>RD1</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดเหนือ)</t>
+          <t>เสาเอ็น คสล. 0.15x0.10 ม. +0.50 ถึง +4.35</t>
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>4</v>
+        <v>146.3</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>24</v>
+        <v>0.57</v>
       </c>
       <c r="G94" s="3" t="n">
-        <v>2.88</v>
+        <v>2.194</v>
       </c>
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>M38</t>
+          <t>M36</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>สมมติขนาด</t>
+          <t>สมมติ: กลางช่วงเสา 6 ม. และข้างวงกบ</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
+          <t>3.2.1 ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>RD2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดใต้)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 +0.50 ถึง +4.35 (ผนังแนวกริด J)</t>
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>4</v>
+        <v>34.65</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>24</v>
+        <v>197.5</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>2.88</v>
+        <v>29.626</v>
       </c>
       <c r="H95" s="3" t="n"/>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>M38</t>
+          <t>M36</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>สมมติขนาด</t>
+          <t>ผู้ว่าจ้างกำหนดระดับ / A202</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>3.4.2 ประตู D1/D2/D4</t>
+          <t>3.2.1 ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>ประตู D1 (ตำแหน่งจาก A101 ขนาดรอตารางประตู)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 +0.50 ถึง +4.35 (ผนังแนวกริด 1)</t>
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>6.3</v>
+        <v>38.5</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>2.77</v>
+        <v>5.77</v>
       </c>
       <c r="G96" s="3" t="n">
-        <v>1.008</v>
+        <v>29.152</v>
       </c>
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="inlineStr">
         <is>
-          <t>M38</t>
+          <t>M36</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101 (ตำแหน่ง) / ขนาดสมมติ</t>
+          <t>ผู้ว่าจ้างกำหนดระดับ / A202</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>3.4.2 ประตู D1/D2/D4</t>
+          <t>3.2.1 ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>ประตู D2 (ตำแหน่งจาก A101 ขนาดรอตารางประตู)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 +0.50 ถึง +4.35 (ผนังแนวกริด 11)</t>
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>4.2</v>
+        <v>38.5</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>7.56</v>
+        <v>5.78</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>1.21</v>
+        <v>29.094</v>
       </c>
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>M38</t>
+          <t>M36</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101 (ตำแหน่ง) / ขนาดสมมติ</t>
+          <t>ผู้ว่าจ้างกำหนดระดับ / A202</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ - ผนังก่ออิฐ</t>
+          <t>ผนังเมทัลชีท (ด้านจั่ว) +5.20 ถึงหลังคา</t>
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>12.52</v>
+        <v>837</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>5.204</v>
+        <v>25.11</v>
       </c>
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M37</t>
         </is>
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
+          <t>แบบ A202</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.1 หลังคาและผนังภายนอก (ผนังเมทัลชีท)</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ - หลังคา/ฝ้า</t>
+          <t>ผนังเมทัลชีท (ด้านชายคา) +5.20 ถึง +10.00</t>
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>19.23</v>
+        <v>0.3</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>1.923</v>
+        <v>16.26</v>
       </c>
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M37</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
+          <t>แบบ A202</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>RD1</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - ผนังก่ออิฐ</t>
+          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดเหนือ)</t>
         </is>
       </c>
       <c r="D100" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E100" s="3" t="n">
-        <v>13.2</v>
-      </c>
       <c r="F100" s="3" t="n">
-        <v>27.16</v>
+        <v>24</v>
       </c>
       <c r="G100" s="3" t="n">
-        <v>6.618</v>
+        <v>2.88</v>
       </c>
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>สมมติขนาด</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4 ประตูม้วน/ประตูเลื่อนขนส่ง</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>RD2</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - หลังคา/ฝ้า</t>
+          <t>ประตูม้วนเหล็ก 6.00x4.00 ม. (ทางลาดใต้)</t>
         </is>
       </c>
       <c r="D101" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>0.1</v>
+        <v>4</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>24.14</v>
+        <v>24</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>2.414</v>
+        <v>2.88</v>
       </c>
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="inlineStr">
         <is>
-          <t>M44</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J101" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>สมมติขนาด</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4.2 ประตู D1/D2/D4</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. - ผนังก่ออิฐ</t>
+          <t>ประตู D1 (ตำแหน่งจาก A101 ขนาดรอตารางประตู)</t>
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>11.2</v>
+        <v>6.3</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>33.77</v>
+        <v>2.77</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>5.001</v>
+        <v>1.008</v>
       </c>
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J102" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>แบบ A101 (ตำแหน่ง) / ขนาดสมมติ</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+          <t>3.4.2 ประตู D1/D2/D4</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. - หลังคา/ฝ้า</t>
+          <t>ประตู D2 (ตำแหน่งจาก A101 ขนาดรอตารางประตู)</t>
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>0.1</v>
+        <v>4.2</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>17.79</v>
+        <v>7.56</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>1.779</v>
+        <v>1.21</v>
       </c>
       <c r="H103" s="3" t="n"/>
       <c r="I103" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>แบบ A101</t>
+          <t>แบบ A101 (ตำแหน่ง) / ขนาดสมมติ</t>
         </is>
       </c>
     </row>
@@ -5781,35 +5781,35 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (รอแบบ) - ผนังก่ออิฐ</t>
+          <t>อาคารห้องน้ำ - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D104" s="3" t="n">
         <v>4</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>11.2</v>
+        <v>10</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>72.63</v>
+        <v>12.52</v>
       </c>
       <c r="G104" s="3" t="n">
-        <v>9.446999999999999</v>
+        <v>5.204</v>
       </c>
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (A101)</t>
+          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
         </is>
       </c>
     </row>
@@ -5821,12 +5821,12 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (รอแบบ) - หลังคา/ฝ้า</t>
+          <t>อาคารห้องน้ำ - หลังคา/ฝ้า</t>
         </is>
       </c>
       <c r="D105" s="3" t="n">
@@ -5836,58 +5836,298 @@
         <v>0.1</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>51.48</v>
+        <v>19.23</v>
       </c>
       <c r="G105" s="3" t="n">
-        <v>5.148</v>
+        <v>1.923</v>
       </c>
       <c r="H105" s="3" t="n"/>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>M39</t>
+          <t>M44</t>
         </is>
       </c>
       <c r="J105" s="3" t="inlineStr">
         <is>
-          <t>สมมติ (A101)</t>
+          <t>สมมติตำแหน่ง/ขนาดจาก A101</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>4.1 งานพื้นถนนรอบอาคาร</t>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>AF01</t>
+          <t>CHEM</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>พื้นทางเท้า/ลานหน้าห้องเก็บสารเคมี AF01</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - ผนังก่ออิฐ</t>
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>0.1</v>
+        <v>13.2</v>
       </c>
       <c r="F106" s="3" t="n">
-        <v>16.74</v>
+        <v>27.16</v>
       </c>
       <c r="G106" s="3" t="n">
-        <v>1.674</v>
+        <v>6.618</v>
       </c>
       <c r="H106" s="3" t="n"/>
       <c r="I106" s="3" t="inlineStr">
         <is>
+          <t>M44</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>แบบ A101</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>CHEM</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. - หลังคา/ฝ้า</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>24.14</v>
+      </c>
+      <c r="G107" s="3" t="n">
+        <v>2.414</v>
+      </c>
+      <c r="H107" s="3" t="n"/>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>M44</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>แบบ A101</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>ห้อง MDB 17.79 ตร.ม. - ผนังก่ออิฐ</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E108" s="3" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>33.77</v>
+      </c>
+      <c r="G108" s="3" t="n">
+        <v>5.001</v>
+      </c>
+      <c r="H108" s="3" t="n"/>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>แบบ A101</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>ห้อง MDB 17.79 ตร.ม. - หลังคา/ฝ้า</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>17.79</v>
+      </c>
+      <c r="G109" s="3" t="n">
+        <v>1.779</v>
+      </c>
+      <c r="H109" s="3" t="n"/>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>แบบ A101</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>ห้องประกอบแนวกริด A (รอแบบ) - ผนังก่ออิฐ</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E110" s="3" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F110" s="3" t="n">
+        <v>72.63</v>
+      </c>
+      <c r="G110" s="3" t="n">
+        <v>9.446999999999999</v>
+      </c>
+      <c r="H110" s="3" t="n"/>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>สมมติ (A101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>3.6 สถาปัตยกรรมอาคารประกอบ</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>ห้องประกอบแนวกริด A (รอแบบ) - หลังคา/ฝ้า</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>51.48</v>
+      </c>
+      <c r="G111" s="3" t="n">
+        <v>5.148</v>
+      </c>
+      <c r="H111" s="3" t="n"/>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>M39</t>
+        </is>
+      </c>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>สมมติ (A101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>4.1 งานพื้นถนนรอบอาคาร</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>AF01</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>พื้นทางเท้า/ลานหน้าห้องเก็บสารเคมี AF01</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F112" s="3" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="G112" s="3" t="n">
+        <v>1.674</v>
+      </c>
+      <c r="H112" s="3" t="n"/>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
           <t>M42</t>
         </is>
       </c>
-      <c r="J106" s="3" t="inlineStr">
+      <c r="J112" s="3" t="inlineStr">
         <is>
           <t>สมมติตำแหน่ง</t>
         </is>
@@ -7119,7 +7359,7 @@
         </is>
       </c>
       <c r="K28" s="3" t="n">
-        <v>6</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29">

</xml_diff>